<commit_message>
feat: implementar la interfaz de usuario de la página de inicio y el componente de navegación global.
</commit_message>
<xml_diff>
--- a/Docs/Cronograma Tienda Online.xlsx
+++ b/Docs/Cronograma Tienda Online.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felipe\Desktop\Tienda online\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5341D8-CEE4-4CD3-93B5-8E6F15A14C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF8B596-023B-4C09-83A4-DD174633FFA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3160,9 +3160,9 @@
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
       <c r="AJ23" s="7"/>
-      <c r="AK23" s="7"/>
+      <c r="AK23" s="6"/>
       <c r="AL23" s="7"/>
-      <c r="AM23" s="7"/>
+      <c r="AM23" s="6"/>
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
@@ -3217,8 +3217,8 @@
       <c r="A24" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>43</v>
+      <c r="B24" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>30</v>
@@ -3693,8 +3693,8 @@
       <c r="A29" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="11" t="s">
-        <v>43</v>
+      <c r="B29" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>50</v>
@@ -3734,7 +3734,7 @@
       <c r="AJ29" s="7"/>
       <c r="AK29" s="7"/>
       <c r="AL29" s="7"/>
-      <c r="AM29" s="7"/>
+      <c r="AM29" s="6"/>
       <c r="AN29" s="7"/>
       <c r="AO29" s="7"/>
       <c r="AP29" s="7"/>

</xml_diff>

<commit_message>
Actualizacion de cronograma y correcion de errores de ui/ux
</commit_message>
<xml_diff>
--- a/Docs/Cronograma Tienda Online.xlsx
+++ b/Docs/Cronograma Tienda Online.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felipe\Desktop\Tienda online\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F644B53-6EEB-4AEF-8156-908B7673864B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358D56D8-B9D9-458F-8E17-C7FEB49D4420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="94">
   <si>
     <t>DIAGRAMA DE GANTT — E-Commerce Felipe Molina | Instituto Tecnológico Sudamericano | Abr 24 – Jul 17, 2026</t>
   </si>
@@ -240,9 +240,6 @@
     <t>Frontend</t>
   </si>
   <si>
-    <t>Pruebas funcionales E2E</t>
-  </si>
-  <si>
     <t>Integración</t>
   </si>
   <si>
@@ -291,9 +288,6 @@
     <t>■ Completado (azul)   ■ Pendiente (naranja)</t>
   </si>
   <si>
-    <t>&lt;</t>
-  </si>
-  <si>
     <t>MAYO</t>
   </si>
   <si>
@@ -310,6 +304,9 @@
   </si>
   <si>
     <t>Config entorno NestJS + PostgreSQL + Prisma</t>
+  </si>
+  <si>
+    <t>Pruebas funcionales</t>
   </si>
 </sst>
 </file>
@@ -997,7 +994,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E2" s="22"/>
       <c r="F2" s="22"/>
@@ -1006,7 +1003,7 @@
       <c r="I2" s="22"/>
       <c r="J2" s="23"/>
       <c r="K2" s="18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L2" s="19"/>
       <c r="M2" s="19"/>
@@ -1039,7 +1036,7 @@
       <c r="AN2" s="19"/>
       <c r="AO2" s="20"/>
       <c r="AP2" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AQ2" s="19"/>
       <c r="AR2" s="19"/>
@@ -1071,7 +1068,7 @@
       <c r="BR2" s="19"/>
       <c r="BS2" s="20"/>
       <c r="BT2" s="24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="BU2" s="22"/>
       <c r="BV2" s="22"/>
@@ -1724,7 +1721,7 @@
     </row>
     <row r="8" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>16</v>
@@ -4716,9 +4713,7 @@
       <c r="V39" s="11"/>
       <c r="W39" s="11"/>
       <c r="X39" s="11"/>
-      <c r="Y39" s="11" t="s">
-        <v>88</v>
-      </c>
+      <c r="Y39" s="11"/>
       <c r="Z39" s="10"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="11"/>
@@ -4784,13 +4779,13 @@
     </row>
     <row r="40" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="11"/>
@@ -4880,13 +4875,13 @@
     </row>
     <row r="41" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D41" s="11"/>
       <c r="E41" s="11"/>
@@ -5260,13 +5255,13 @@
     </row>
     <row r="45" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D45" s="11"/>
       <c r="E45" s="11"/>
@@ -5356,13 +5351,13 @@
     </row>
     <row r="46" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="12"/>
@@ -5452,7 +5447,7 @@
     </row>
     <row r="47" spans="1:88" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
@@ -5544,13 +5539,13 @@
     </row>
     <row r="48" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D48" s="12"/>
       <c r="E48" s="12"/>
@@ -5640,13 +5635,13 @@
     </row>
     <row r="49" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
@@ -5735,7 +5730,7 @@
     </row>
     <row r="50" spans="1:88" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -5827,13 +5822,13 @@
     </row>
     <row r="51" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D51" s="11"/>
       <c r="E51" s="11"/>
@@ -5923,13 +5918,13 @@
     </row>
     <row r="52" spans="1:88" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D52" s="12"/>
       <c r="E52" s="12"/>
@@ -6019,7 +6014,7 @@
     </row>
     <row r="54" spans="1:88" x14ac:dyDescent="0.3">
       <c r="A54" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>

</xml_diff>